<commit_message>
Fix sample_data.xlsx to be a valid Excel file
Regenerate via pandas/openpyxl instead of a hand-built minimal XLSX,
which Excel flagged for repair due to missing standard parts.
</commit_message>
<xml_diff>
--- a/data/sample_data.xlsx
+++ b/data/sample_data.xlsx
@@ -1,23 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
       <sz val="11"/>
-      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="1">
+  <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
@@ -33,14 +47,374 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  </cellStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
+</file>
+
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -92,7 +466,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Women in Trade Initiative</t>
+          <t>Ghana Youth Enterprise Fund</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -102,40 +476,40 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Ashanti</t>
+          <t>Greater Accra</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Growth</t>
-        </is>
-      </c>
-      <c r="F2">
-        <v>2</v>
-      </c>
-      <c r="G2">
-        <v>27.2</v>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>8</v>
+      </c>
+      <c r="G2" t="n">
+        <v>7.1</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2023-10-15</t>
+          <t>2023-10-13</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Grant</t>
+          <t>Loan</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Northern Region Agribusiness Accelerator</t>
+          <t>Volta Delta Enterprise Hub</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -150,35 +524,35 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Northern</t>
+          <t>Greater Accra</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Growth</t>
-        </is>
-      </c>
-      <c r="F3">
-        <v>4</v>
-      </c>
-      <c r="G3">
-        <v>25.3</v>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-3.4</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2024-02-22</t>
+          <t>2024-04-21</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Grant</t>
+          <t>Loan</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Volta Delta Enterprise Hub</t>
+          <t>Ghana Youth Enterprise Fund</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -188,33 +562,33 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>Upper East</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Growth</t>
-        </is>
-      </c>
-      <c r="F4">
-        <v>6</v>
-      </c>
-      <c r="G4">
-        <v>0.1</v>
+          <t>Startup</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>13</v>
+      </c>
+      <c r="G4" t="n">
+        <v>5.4</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2025-02-11</t>
+          <t>2024-07-23</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Grant</t>
+          <t>Equipment</t>
         </is>
       </c>
     </row>
@@ -236,35 +610,35 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Ashanti</t>
+          <t>Western</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Startup</t>
-        </is>
-      </c>
-      <c r="F5">
-        <v>14</v>
-      </c>
-      <c r="G5">
-        <v>39.5</v>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G5" t="n">
+        <v>5.1</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2023-07-24</t>
+          <t>2024-11-20</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Mentorship</t>
+          <t>Equipment</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Northern Region Agribusiness Accelerator</t>
+          <t>Ghana Youth Enterprise Fund</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -274,37 +648,38 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Greater Accra</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Idea</t>
-        </is>
-      </c>
-      <c r="G6">
-        <v>28.8</v>
+          <t>Mature</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="n">
+        <v>49.3</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2025-03-30</t>
+          <t>2024-06-25</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Grant</t>
+          <t>Loan</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Northern Region Agribusiness Accelerator</t>
+          <t>Volta Delta Enterprise Hub</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -319,23 +694,23 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Bono</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Growth</t>
-        </is>
-      </c>
-      <c r="F7">
-        <v>10</v>
-      </c>
-      <c r="G7">
-        <v>-1.8</v>
+          <t>Startup</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G7" t="n">
+        <v>28.6</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2025-04-25</t>
+          <t>2025-01-10</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -347,7 +722,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Women in Trade Initiative</t>
+          <t>Ghana Youth Enterprise Fund</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -362,35 +737,35 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Volta</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Idea</t>
-        </is>
-      </c>
-      <c r="F8">
-        <v>8</v>
-      </c>
-      <c r="G8">
-        <v>-6.6</v>
+          <t>Mature</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>9</v>
+      </c>
+      <c r="G8" t="n">
+        <v>59</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2025-02-12</t>
+          <t>2024-04-21</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Grant</t>
+          <t>Mentorship</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Ghana Youth Enterprise Fund</t>
+          <t>GrowGhana SME Support</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -400,12 +775,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Northern</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -413,24 +788,25 @@
           <t>Startup</t>
         </is>
       </c>
-      <c r="F9">
-        <v>1</v>
-      </c>
+      <c r="F9" t="n">
+        <v>5</v>
+      </c>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2025-02-25</t>
+          <t>2025-01-28</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Grant</t>
+          <t>Mentorship</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Ghana Youth Enterprise Fund</t>
+          <t>Northern Region Agribusiness Accelerator</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -440,40 +816,40 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Western</t>
+          <t>Upper West</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Idea</t>
-        </is>
-      </c>
-      <c r="F10">
-        <v>8</v>
-      </c>
-      <c r="G10">
-        <v>25</v>
+          <t>Mature</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>5</v>
+      </c>
+      <c r="G10" t="n">
+        <v>27.4</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2025-06-26</t>
+          <t>2024-05-16</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Grant</t>
+          <t>Equipment</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Women in Trade Initiative</t>
+          <t>Northern Region Agribusiness Accelerator</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -488,7 +864,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Greater Accra</t>
+          <t>Upper East</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -496,27 +872,27 @@
           <t>Idea</t>
         </is>
       </c>
-      <c r="F11">
-        <v>14</v>
-      </c>
-      <c r="G11">
-        <v>55.5</v>
+      <c r="F11" t="n">
+        <v>7</v>
+      </c>
+      <c r="G11" t="n">
+        <v>37.9</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2024-02-15</t>
+          <t>2023-04-25</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Mentorship</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Volta Delta Enterprise Hub</t>
+          <t>Northern Region Agribusiness Accelerator</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -526,7 +902,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -536,18 +912,18 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Growth</t>
-        </is>
-      </c>
-      <c r="F12">
-        <v>12</v>
-      </c>
-      <c r="G12">
-        <v>27.4</v>
+          <t>Mature</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>2</v>
+      </c>
+      <c r="G12" t="n">
+        <v>4.8</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2023-11-22</t>
+          <t>2024-10-06</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -559,7 +935,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Ghana Youth Enterprise Fund</t>
+          <t>Volta Delta Enterprise Hub</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -574,35 +950,35 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Greater Accra</t>
+          <t>Bono</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Idea</t>
-        </is>
-      </c>
-      <c r="F13">
-        <v>14</v>
-      </c>
-      <c r="G13">
-        <v>57.3</v>
+          <t>Growth</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>4</v>
+      </c>
+      <c r="G13" t="n">
+        <v>8.5</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2025-02-17</t>
+          <t>2024-05-20</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Mentorship</t>
+          <t>Loan</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>GrowGhana SME Support</t>
+          <t>Volta Delta Enterprise Hub</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -612,12 +988,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Bono</t>
+          <t>Upper West</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -625,27 +1001,27 @@
           <t>Mature</t>
         </is>
       </c>
-      <c r="F14">
-        <v>2</v>
-      </c>
-      <c r="G14">
-        <v>-0.8</v>
+      <c r="F14" t="n">
+        <v>12</v>
+      </c>
+      <c r="G14" t="n">
+        <v>15.3</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2024-10-09</t>
+          <t>2023-10-11</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Equipment</t>
+          <t>Grant</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Ghana Youth Enterprise Fund</t>
+          <t>Volta Delta Enterprise Hub</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -655,33 +1031,33 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Bono</t>
+          <t>Ashanti</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Startup</t>
-        </is>
-      </c>
-      <c r="F15">
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
         <v>4</v>
       </c>
-      <c r="G15">
-        <v>30</v>
+      <c r="G15" t="n">
+        <v>33.9</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2024-12-13</t>
+          <t>2025-05-14</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Loan</t>
+          <t>Equipment</t>
         </is>
       </c>
     </row>
@@ -698,25 +1074,26 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Northern</t>
+          <t>Upper West</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Startup</t>
-        </is>
-      </c>
-      <c r="G16">
-        <v>8</v>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="n">
+        <v>59.7</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2023-08-25</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -728,7 +1105,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Volta Delta Enterprise Hub</t>
+          <t>Women in Trade Initiative</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -743,7 +1120,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Ashanti</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -751,27 +1128,27 @@
           <t>Idea</t>
         </is>
       </c>
-      <c r="F17">
-        <v>1</v>
-      </c>
-      <c r="G17">
-        <v>12.3</v>
+      <c r="F17" t="n">
+        <v>3</v>
+      </c>
+      <c r="G17" t="n">
+        <v>10.5</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2025-04-02</t>
+          <t>2023-11-20</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Grant</t>
+          <t>Mentorship</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>GrowGhana SME Support</t>
+          <t>Volta Delta Enterprise Hub</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -781,7 +1158,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -791,30 +1168,30 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Growth</t>
-        </is>
-      </c>
-      <c r="F18">
+          <t>Startup</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
         <v>3</v>
       </c>
-      <c r="G18">
-        <v>55.8</v>
+      <c r="G18" t="n">
+        <v>50.9</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2023-11-02</t>
+          <t>2024-09-03</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Equipment</t>
+          <t>Training</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Northern Region Agribusiness Accelerator</t>
+          <t>Women in Trade Initiative</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -824,7 +1201,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -834,27 +1211,28 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Mature</t>
-        </is>
-      </c>
-      <c r="F19">
-        <v>2</v>
-      </c>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2023-02-02</t>
+          <t>2024-10-25</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Loan</t>
+          <t>Grant</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>GrowGhana SME Support</t>
+          <t>Ghana Youth Enterprise Fund</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -869,23 +1247,23 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Ashanti</t>
+          <t>Western</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Growth</t>
-        </is>
-      </c>
-      <c r="F20">
-        <v>14</v>
-      </c>
-      <c r="G20">
-        <v>3.3</v>
+          <t>Mature</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>7</v>
+      </c>
+      <c r="G20" t="n">
+        <v>-5.9</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2024-09-05</t>
+          <t>2023-06-11</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -897,7 +1275,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Volta Delta Enterprise Hub</t>
+          <t>GrowGhana SME Support</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -907,35 +1285,36 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Female</t>
-        </is>
-      </c>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Startup</t>
-        </is>
-      </c>
-      <c r="F21">
-        <v>6</v>
-      </c>
-      <c r="G21">
-        <v>52.4</v>
+          <t>Mature</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>4</v>
+      </c>
+      <c r="G21" t="n">
+        <v>36.2</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2024-01-17</t>
+          <t>2023-12-05</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Mentorship</t>
+          <t>Training</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Volta Delta Enterprise Hub</t>
+          <t>Women in Trade Initiative</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -945,40 +1324,40 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Upper East</t>
+          <t>Western</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Growth</t>
-        </is>
-      </c>
-      <c r="F22">
-        <v>2</v>
-      </c>
-      <c r="G22">
-        <v>-3</v>
+          <t>Mature</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>12</v>
+      </c>
+      <c r="G22" t="n">
+        <v>59.7</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>2023-07-19</t>
+          <t>2025-02-03</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Mentorship</t>
+          <t>Grant</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ghana Youth Enterprise Fund</t>
+          <t>Volta Delta Enterprise Hub</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -988,12 +1367,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Western</t>
+          <t>Volta</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1001,20 +1380,20 @@
           <t>Startup</t>
         </is>
       </c>
-      <c r="F23">
-        <v>1</v>
-      </c>
-      <c r="G23">
-        <v>55</v>
+      <c r="F23" t="n">
+        <v>2</v>
+      </c>
+      <c r="G23" t="n">
+        <v>13.7</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2025-09-02</t>
+          <t>2024-04-16</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Mentorship</t>
+          <t>Grant</t>
         </is>
       </c>
     </row>
@@ -1031,40 +1410,40 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Upper West</t>
+          <t>Greater Accra</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Mature</t>
-        </is>
-      </c>
-      <c r="F24">
-        <v>13</v>
-      </c>
-      <c r="G24">
-        <v>43.3</v>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>7</v>
+      </c>
+      <c r="G24" t="n">
+        <v>-5.3</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>2024-01-07</t>
+          <t>2023-03-06</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Loan</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Women in Trade Initiative</t>
+          <t>Volta Delta Enterprise Hub</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1074,40 +1453,40 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Western</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Idea</t>
-        </is>
-      </c>
-      <c r="F25">
-        <v>3</v>
-      </c>
-      <c r="G25">
-        <v>9.2</v>
+          <t>Mature</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>15</v>
+      </c>
+      <c r="G25" t="n">
+        <v>5</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>2025-07-01</t>
+          <t>2023-09-28</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Mentorship</t>
+          <t>Training</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>GrowGhana SME Support</t>
+          <t>Women in Trade Initiative</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1122,25 +1501,26 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Upper East</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Mature</t>
-        </is>
-      </c>
-      <c r="G26">
-        <v>46</v>
+          <t>Growth</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="n">
+        <v>3.3</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>2025-10-29</t>
+          <t>2023-07-18</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Loan</t>
+          <t>Equipment</t>
         </is>
       </c>
     </row>
@@ -1157,12 +1537,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>Bono</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1170,27 +1550,27 @@
           <t>Mature</t>
         </is>
       </c>
-      <c r="F27">
-        <v>3</v>
-      </c>
-      <c r="G27">
-        <v>35.5</v>
+      <c r="F27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" t="n">
+        <v>37.1</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>2025-02-14</t>
+          <t>2023-07-21</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Mentorship</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Ghana Youth Enterprise Fund</t>
+          <t>Northern Region Agribusiness Accelerator</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1200,12 +1580,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Bono</t>
+          <t>Volta</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1213,27 +1593,27 @@
           <t>Mature</t>
         </is>
       </c>
-      <c r="F28">
-        <v>3</v>
-      </c>
-      <c r="G28">
-        <v>27.8</v>
+      <c r="F28" t="n">
+        <v>6</v>
+      </c>
+      <c r="G28" t="n">
+        <v>3.3</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>2024-09-29</t>
+          <t>2025-07-07</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Grant</t>
+          <t>Training</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Northern Region Agribusiness Accelerator</t>
+          <t>Women in Trade Initiative</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1243,37 +1623,38 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Northern</t>
+          <t>Bono</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Startup</t>
-        </is>
-      </c>
-      <c r="F29">
-        <v>5</v>
-      </c>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>7</v>
+      </c>
+      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
-          <t>2023-07-07</t>
+          <t>2023-06-04</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Loan</t>
+          <t>Grant</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Northern Region Agribusiness Accelerator</t>
+          <t>Women in Trade Initiative</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1288,35 +1669,35 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Volta</t>
+          <t>Ashanti</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Mature</t>
-        </is>
-      </c>
-      <c r="F30">
+          <t>Startup</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
         <v>7</v>
       </c>
-      <c r="G30">
-        <v>44.7</v>
+      <c r="G30" t="n">
+        <v>1.6</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-09-21</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Equipment</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Ghana Youth Enterprise Fund</t>
+          <t>GrowGhana SME Support</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1331,35 +1712,35 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Upper West</t>
+          <t>Northern</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Startup</t>
-        </is>
-      </c>
-      <c r="F31">
-        <v>9</v>
-      </c>
-      <c r="G31">
-        <v>33.4</v>
+          <t>Mature</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>12</v>
+      </c>
+      <c r="G31" t="n">
+        <v>-9.800000000000001</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>2025-11-12</t>
+          <t>2025-03-10</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Loan</t>
+          <t>Mentorship</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>GrowGhana SME Support</t>
+          <t>Northern Region Agribusiness Accelerator</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1369,12 +1750,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Upper West</t>
+          <t>Upper East</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1382,15 +1763,15 @@
           <t>Idea</t>
         </is>
       </c>
-      <c r="F32">
-        <v>14</v>
-      </c>
-      <c r="G32">
-        <v>53</v>
+      <c r="F32" t="n">
+        <v>15</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0.8</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>2023-11-23</t>
+          <t>2024-08-30</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -1402,7 +1783,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Women in Trade Initiative</t>
+          <t>Volta Delta Enterprise Hub</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1417,35 +1798,35 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Idea</t>
-        </is>
-      </c>
-      <c r="F33">
-        <v>10</v>
-      </c>
-      <c r="G33">
-        <v>59.3</v>
+          <t>Startup</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" t="n">
+        <v>-6.5</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>2025-10-26</t>
+          <t>2025-09-03</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Grant</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Northern Region Agribusiness Accelerator</t>
+          <t>Women in Trade Initiative</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1455,40 +1836,40 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Greater Accra</t>
+          <t>Northern</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Growth</t>
-        </is>
-      </c>
-      <c r="F34">
-        <v>10</v>
-      </c>
-      <c r="G34">
-        <v>27.4</v>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>2</v>
+      </c>
+      <c r="G34" t="n">
+        <v>31.7</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>2024-01-12</t>
+          <t>2024-04-26</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Equipment</t>
+          <t>Loan</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Northern Region Agribusiness Accelerator</t>
+          <t>Volta Delta Enterprise Hub</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1498,40 +1879,40 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Volta</t>
+          <t>Upper West</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Mature</t>
-        </is>
-      </c>
-      <c r="F35">
-        <v>10</v>
-      </c>
-      <c r="G35">
-        <v>-2.9</v>
+          <t>Growth</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" t="n">
+        <v>33.4</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>2025-07-11</t>
+          <t>2025-05-08</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Mentorship</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Women in Trade Initiative</t>
+          <t>Northern Region Agribusiness Accelerator</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1551,27 +1932,28 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Idea</t>
-        </is>
-      </c>
-      <c r="G36">
-        <v>14.2</v>
+          <t>Growth</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="n">
+        <v>6.7</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>2023-07-20</t>
+          <t>2025-03-21</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Loan</t>
+          <t>Equipment</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Northern Region Agribusiness Accelerator</t>
+          <t>Ghana Youth Enterprise Fund</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1581,33 +1963,33 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Ashanti</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Growth</t>
-        </is>
-      </c>
-      <c r="F37">
-        <v>3</v>
-      </c>
-      <c r="G37">
-        <v>35.7</v>
+          <t>Startup</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" t="n">
+        <v>22.1</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>2025-07-31</t>
+          <t>2023-07-24</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Mentorship</t>
+          <t>Loan</t>
         </is>
       </c>
     </row>
@@ -1624,12 +2006,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Ashanti</t>
+          <t>Northern</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1637,27 +2019,27 @@
           <t>Growth</t>
         </is>
       </c>
-      <c r="F38">
-        <v>12</v>
-      </c>
-      <c r="G38">
-        <v>29.5</v>
+      <c r="F38" t="n">
+        <v>11</v>
+      </c>
+      <c r="G38" t="n">
+        <v>51.7</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>2025-01-06</t>
+          <t>2024-05-15</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Loan</t>
+          <t>Training</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Volta Delta Enterprise Hub</t>
+          <t>Ghana Youth Enterprise Fund</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1672,7 +2054,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Northern</t>
+          <t>Upper East</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1680,24 +2062,25 @@
           <t>Growth</t>
         </is>
       </c>
-      <c r="F39">
-        <v>4</v>
-      </c>
+      <c r="F39" t="n">
+        <v>9</v>
+      </c>
+      <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
-          <t>2024-08-14</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Grant</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Ghana Youth Enterprise Fund</t>
+          <t>GrowGhana SME Support</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1707,40 +2090,40 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Bono</t>
+          <t>Western</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Startup</t>
-        </is>
-      </c>
-      <c r="F40">
-        <v>7</v>
-      </c>
-      <c r="G40">
-        <v>60.5</v>
+          <t>Growth</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>3</v>
+      </c>
+      <c r="G40" t="n">
+        <v>52.3</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>2025-07-30</t>
+          <t>2023-11-15</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Mentorship</t>
+          <t>Loan</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Northern Region Agribusiness Accelerator</t>
+          <t>Volta Delta Enterprise Hub</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1760,30 +2143,30 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Startup</t>
-        </is>
-      </c>
-      <c r="F41">
+          <t>Mature</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
         <v>6</v>
       </c>
-      <c r="G41">
-        <v>-9</v>
+      <c r="G41" t="n">
+        <v>38.1</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>2024-05-20</t>
+          <t>2024-06-24</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Equipment</t>
+          <t>Mentorship</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Volta Delta Enterprise Hub</t>
+          <t>Ghana Youth Enterprise Fund</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1798,7 +2181,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Greater Accra</t>
+          <t>Ashanti</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1806,15 +2189,15 @@
           <t>Growth</t>
         </is>
       </c>
-      <c r="F42">
-        <v>3</v>
-      </c>
-      <c r="G42">
-        <v>46.5</v>
+      <c r="F42" t="n">
+        <v>13</v>
+      </c>
+      <c r="G42" t="n">
+        <v>48.1</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>2025-09-20</t>
+          <t>2023-04-01</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -1826,7 +2209,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Northern Region Agribusiness Accelerator</t>
+          <t>Volta Delta Enterprise Hub</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1841,7 +2224,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Upper East</t>
+          <t>Northern</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -1849,15 +2232,15 @@
           <t>Idea</t>
         </is>
       </c>
-      <c r="F43">
-        <v>10</v>
-      </c>
-      <c r="G43">
-        <v>35.8</v>
+      <c r="F43" t="n">
+        <v>14</v>
+      </c>
+      <c r="G43" t="n">
+        <v>28.6</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>2024-07-07</t>
+          <t>2025-05-25</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -1869,7 +2252,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Ghana Youth Enterprise Fund</t>
+          <t>Women in Trade Initiative</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1879,12 +2262,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Northern</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -1892,15 +2275,15 @@
           <t>Startup</t>
         </is>
       </c>
-      <c r="F44">
-        <v>14</v>
-      </c>
-      <c r="G44">
-        <v>30.2</v>
+      <c r="F44" t="n">
+        <v>1</v>
+      </c>
+      <c r="G44" t="n">
+        <v>48.4</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>2024-02-18</t>
+          <t>2023-10-31</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -1912,7 +2295,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Volta Delta Enterprise Hub</t>
+          <t>Northern Region Agribusiness Accelerator</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1922,25 +2305,28 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Startup</t>
-        </is>
-      </c>
-      <c r="G45">
-        <v>6.9</v>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>1</v>
+      </c>
+      <c r="G45" t="n">
+        <v>52.9</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>2025-06-24</t>
+          <t>2024-03-06</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -1952,7 +2338,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Ghana Youth Enterprise Fund</t>
+          <t>Northern Region Agribusiness Accelerator</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1962,37 +2348,38 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Bono</t>
+          <t>Upper West</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Growth</t>
-        </is>
-      </c>
-      <c r="G46">
-        <v>10.5</v>
+          <t>Startup</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="n">
+        <v>42.5</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>2023-02-24</t>
+          <t>2024-04-29</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Grant</t>
+          <t>Equipment</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Volta Delta Enterprise Hub</t>
+          <t>Northern Region Agribusiness Accelerator</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2002,40 +2389,40 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Bono</t>
+          <t>Northern</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Startup</t>
-        </is>
-      </c>
-      <c r="F47">
-        <v>8</v>
-      </c>
-      <c r="G47">
-        <v>41.9</v>
+          <t>Growth</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>10</v>
+      </c>
+      <c r="G47" t="n">
+        <v>44.8</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>2025-01-11</t>
+          <t>2025-04-23</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Mentorship</t>
+          <t>Training</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Ghana Youth Enterprise Fund</t>
+          <t>Northern Region Agribusiness Accelerator</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2045,12 +2432,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Bono</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2058,27 +2445,27 @@
           <t>Mature</t>
         </is>
       </c>
-      <c r="F48">
-        <v>13</v>
-      </c>
-      <c r="G48">
-        <v>56.8</v>
+      <c r="F48" t="n">
+        <v>1</v>
+      </c>
+      <c r="G48" t="n">
+        <v>50.1</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>2024-12-26</t>
+          <t>2024-03-31</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Loan</t>
+          <t>Mentorship</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Volta Delta Enterprise Hub</t>
+          <t>Northern Region Agribusiness Accelerator</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2093,7 +2480,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Ashanti</t>
+          <t>Volta</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2101,12 +2488,13 @@
           <t>Mature</t>
         </is>
       </c>
-      <c r="F49">
-        <v>11</v>
-      </c>
+      <c r="F49" t="n">
+        <v>7</v>
+      </c>
+      <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2023-02-18</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -2118,7 +2506,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Volta Delta Enterprise Hub</t>
+          <t>Women in Trade Initiative</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2138,18 +2526,18 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Mature</t>
-        </is>
-      </c>
-      <c r="F50">
-        <v>4</v>
-      </c>
-      <c r="G50">
-        <v>48.4</v>
+          <t>Growth</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>8</v>
+      </c>
+      <c r="G50" t="n">
+        <v>14.6</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>2024-09-21</t>
+          <t>2025-11-09</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -2171,36 +2559,37 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Volta</t>
+          <t>Western</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Mature</t>
-        </is>
-      </c>
-      <c r="F51">
-        <v>13</v>
-      </c>
-      <c r="G51">
-        <v>17.1</v>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>5</v>
+      </c>
+      <c r="G51" t="n">
+        <v>30.6</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2024-06-27</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Mentorship</t>
+          <t>Loan</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>